<commit_message>
Always Pro; login errors; signup name/org; progress UX; trial request form
</commit_message>
<xml_diff>
--- a/Feedbacks.xlsx
+++ b/Feedbacks.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Rony\Desktop\transcriber\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{418C26E9-63F6-458A-8E3E-8E748723296E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3E8E8E4E-D7A2-4128-94B2-5E0D0DB3C440}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -33,6 +33,32 @@
     </ext>
   </extLst>
 </workbook>
+</file>
+
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7" uniqueCount="7">
+  <si>
+    <t>Feedbacks and feature requests</t>
+  </si>
+  <si>
+    <t>First of all the we have deployed our website at https://web-production-d958a.up.railway.app/</t>
+  </si>
+  <si>
+    <t>I have given to one email 5 mins, then using that mail I have logged in and then uploaded audio for transcription. After these from then to now I can see it showing status is pending. Also, my api already charged around 0.22 I can see from my google studio, but transcription was not given. Also, from admin panel I can see job status for that email is pending and model named flashed. but instead of flash I want to always use pro. Also, as we dont have any free trail so please remove free trail from entire website. Additionally, keep one form for those people who wants to get a trail, We will collect those responses and give them some credits</t>
+  </si>
+  <si>
+    <t xml:space="preserve">When the audio file uploaded and it shows processing or pending or in future it might be completed, its showing that the page will automatically update, when transcription is done, its look too generic, user don’t know when it will be done, how much time it will take, and when they will get their output. So, this issue needs to be consider. </t>
+  </si>
+  <si>
+    <t>In user signup there could be some sort of information like Name email organisation name (optional) things etc. also when trying to login, If I put wrong things it should be shown wrong username or password.</t>
+  </si>
+  <si>
+    <t>Also, if all things are okay, I want to deploy on custom domain name</t>
+  </si>
+  <si>
+    <t>whatsapp number - 01772215084 Bkash number- 01575522637</t>
+  </si>
+</sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
@@ -348,12 +374,48 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1"/>
+  <dimension ref="A1:A7"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="19.5546875" customWidth="1"/>
   </cols>
-  <sheetData/>
+  <sheetData>
+    <row r="1" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="2" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="4" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="5" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="6" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="7" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
+        <v>6</v>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>